<commit_message>
Kotoba1 v1.0.3: quiz audio text corrections
- ERABE No23: 花火は→TTS, text display fix
- ERABE No45: タンバリン audio update
- ERABE No46: クレヨン audio update
- ERABE No47: 鉛筆は→TTS, text display fix

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Kotoba1/quiz-mondai-an.xlsx
+++ b/Kotoba1/quiz-mondai-an.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ygami_data\DevWorks\aiay-lab-kids-app\Kotoba1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B993317D-5CC1-4E8C-8218-2E2455294524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{092FD149-1037-4FC4-AB96-4AF86ED43156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29580" yWindow="765" windowWidth="21600" windowHeight="11175" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ならべるクイズ" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="714" uniqueCount="283">
   <si>
     <t>No</t>
   </si>
@@ -822,10 +822,6 @@
   </si>
   <si>
     <t>描画道具の識別</t>
-  </si>
-  <si>
-    <t>たんばりんをたたくのは どっち？</t>
-    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>しんごうをまつ</t>
@@ -844,10 +840,6 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>くれよんでは どっち？</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>えんぴつは どっち？</t>
     <phoneticPr fontId="2"/>
   </si>
@@ -877,6 +869,28 @@
   </si>
   <si>
     <t>せんがほそいのは どっち？</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>花火は どっち？</t>
+    <rPh sb="0" eb="2">
+      <t>ハナビ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>鉛筆は どっち？</t>
+    <rPh sb="0" eb="2">
+      <t>エンピツ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>クレヨンは どっち？</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>タンバリンをたたくのは どっち？</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -2739,13 +2753,13 @@
         <v>109</v>
       </c>
       <c r="C53" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="D53" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E53" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="F53">
         <v>5</v>
@@ -2944,7 +2958,7 @@
         <v>137</v>
       </c>
       <c r="C61" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D61" t="s">
         <v>138</v>
@@ -3100,13 +3114,13 @@
         <v>130</v>
       </c>
       <c r="C67" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D67" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="E67" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="F67">
         <v>6</v>
@@ -3126,13 +3140,13 @@
         <v>261</v>
       </c>
       <c r="C68" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D68" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E68" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F68">
         <v>6</v>
@@ -3716,6 +3730,9 @@
         <v>19</v>
       </c>
       <c r="F24" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>224</v>
       </c>
       <c r="H24" s="2" t="s">
@@ -4109,7 +4126,7 @@
         <v>143</v>
       </c>
       <c r="F42" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H42" t="s">
         <v>258</v>
@@ -4149,13 +4166,13 @@
         <v>261</v>
       </c>
       <c r="D44" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="E44" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F44" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H44" t="s">
         <v>262</v>
@@ -4201,7 +4218,7 @@
         <v>139</v>
       </c>
       <c r="F46" t="s">
-        <v>267</v>
+        <v>282</v>
       </c>
       <c r="H46" t="s">
         <v>265</v>
@@ -4224,7 +4241,7 @@
         <v>145</v>
       </c>
       <c r="F47" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="H47" t="s">
         <v>266</v>
@@ -4247,7 +4264,10 @@
         <v>144</v>
       </c>
       <c r="F48" t="s">
-        <v>273</v>
+        <v>280</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>271</v>
       </c>
       <c r="H48" t="s">
         <v>266</v>
@@ -4264,13 +4284,13 @@
         <v>130</v>
       </c>
       <c r="D49" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E49" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="F49" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.15">
@@ -4290,7 +4310,7 @@
         <v>145</v>
       </c>
       <c r="F50" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.15">
@@ -4310,7 +4330,7 @@
         <v>144</v>
       </c>
       <c r="F51" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.15">
@@ -4330,7 +4350,7 @@
         <v>144</v>
       </c>
       <c r="F52" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.15">
@@ -4350,7 +4370,7 @@
         <v>145</v>
       </c>
       <c r="F53" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Kotoba1 v1.0.6: erabe UX fixes, quiz data update, SVG handrail
- Fix score double-counting when using back button (scoredSet)
- Add No.54 (waiting-crosswalk-cars) and No.55 (te-wo-fuku) quiz entries
- Reorder home menu: えをえらぶ above ならべる
- Add handrail post at bottom step in kaidan SVGs

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Kotoba1/quiz-mondai-an.xlsx
+++ b/Kotoba1/quiz-mondai-an.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ygami_data\DevWorks\aiay-lab-kids-app\Kotoba1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31639D32-4838-4DC5-83D1-5B2299A83DAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D948AD00-E83E-448B-9D69-D86F5FDEBC8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ならべるクイズ" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="289">
   <si>
     <t>No</t>
   </si>
@@ -602,12 +602,6 @@
     <t>ねる</t>
   </si>
   <si>
-    <t>おきるのは どっち？</t>
-  </si>
-  <si>
-    <t>ねるのは どっち？</t>
-  </si>
-  <si>
     <t>まどをしめるのは どっち？</t>
   </si>
   <si>
@@ -647,9 +641,6 @@
     <t>しんごうをまつ</t>
   </si>
   <si>
-    <t>わたるのはどっち？</t>
-  </si>
-  <si>
     <t>渡る↔待つの対比</t>
   </si>
   <si>
@@ -875,7 +866,35 @@
     <t>たんばりん</t>
   </si>
   <si>
-    <t>あり</t>
+    <t>ねているのは どっち？</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>おきたのは どっち？</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>あかしんごうは どっち？</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>てを ふくのは どっち？</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>あおしんごうはどっち？</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>kaidan-wo-noboru.svg</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>kaidan-wo-oriru.svg</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>あめが ふるのは どっち？</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -1399,22 +1418,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
@@ -1425,25 +1444,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="F2" s="6">
         <v>2</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1466,10 +1485,10 @@
         <v>2</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1480,22 +1499,22 @@
         <v>63</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="F4" s="6">
         <v>2</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1506,22 +1525,22 @@
         <v>64</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="F5" s="7">
         <v>2</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1544,10 +1563,10 @@
         <v>2</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1558,22 +1577,22 @@
         <v>105</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="F7" s="7">
         <v>2</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1596,10 +1615,10 @@
         <v>2</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1622,10 +1641,10 @@
         <v>3</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1648,10 +1667,10 @@
         <v>3</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1674,10 +1693,10 @@
         <v>3</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1688,22 +1707,22 @@
         <v>130</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>131</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="F12" s="6">
         <v>3</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1726,10 +1745,10 @@
         <v>3</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1740,22 +1759,22 @@
         <v>51</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="F14" s="6">
         <v>3</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1766,22 +1785,22 @@
         <v>106</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="F15" s="7">
         <v>3</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1804,10 +1823,10 @@
         <v>4</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1830,10 +1849,10 @@
         <v>4</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1856,10 +1875,10 @@
         <v>4</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1870,22 +1889,22 @@
         <v>112</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F19" s="9">
         <v>4</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1908,10 +1927,10 @@
         <v>4</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1922,22 +1941,22 @@
         <v>88</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>90</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="F21" s="9">
         <v>4</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1948,22 +1967,22 @@
         <v>45</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="F22" s="8">
         <v>4</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -1974,22 +1993,22 @@
         <v>46</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="F23" s="9">
         <v>4</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -2000,22 +2019,22 @@
         <v>40</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="F24" s="8">
         <v>4</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -2026,22 +2045,22 @@
         <v>39</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="F25" s="9">
         <v>4</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -2052,22 +2071,22 @@
         <v>70</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F26" s="8">
         <v>4</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -2090,10 +2109,10 @@
         <v>5</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -2104,22 +2123,22 @@
         <v>119</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="F28" s="11">
         <v>7</v>
       </c>
       <c r="G28" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="H28" s="11" t="s">
         <v>262</v>
-      </c>
-      <c r="H28" s="11" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -2142,10 +2161,10 @@
         <v>5</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -2162,16 +2181,16 @@
         <v>127</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="F30" s="11">
         <v>5</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -2194,10 +2213,10 @@
         <v>6</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
@@ -2220,10 +2239,10 @@
         <v>6</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.15">
@@ -2246,10 +2265,10 @@
         <v>8</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.15">
@@ -2272,10 +2291,10 @@
         <v>6</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.15">
@@ -2308,10 +2327,10 @@
         <v>6</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.15">
@@ -2334,10 +2353,10 @@
         <v>5</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.15">
@@ -2360,10 +2379,10 @@
         <v>6</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H38" s="14" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.15">
@@ -2386,10 +2405,10 @@
         <v>6</v>
       </c>
       <c r="G39" s="13" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.15">
@@ -2412,10 +2431,10 @@
         <v>7</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H40" s="14" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.15">
@@ -2438,10 +2457,10 @@
         <v>8</v>
       </c>
       <c r="G41" s="13" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H41" s="13" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.15">
@@ -2464,10 +2483,10 @@
         <v>6</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H42" s="14" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.15">
@@ -2490,10 +2509,10 @@
         <v>6</v>
       </c>
       <c r="G43" s="13" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H43" s="13" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.15">
@@ -2516,10 +2535,10 @@
         <v>2</v>
       </c>
       <c r="G44" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H44" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.15">
@@ -2542,10 +2561,10 @@
         <v>3</v>
       </c>
       <c r="G45" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H45" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.15">
@@ -2556,22 +2575,22 @@
         <v>156</v>
       </c>
       <c r="C46" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="D46" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="E46" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="F46">
         <v>3</v>
       </c>
       <c r="G46" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H46" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.15">
@@ -2582,22 +2601,22 @@
         <v>168</v>
       </c>
       <c r="C47" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D47" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="E47" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="F47">
         <v>4</v>
       </c>
       <c r="G47" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H47" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.15">
@@ -2608,22 +2627,22 @@
         <v>173</v>
       </c>
       <c r="C48" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D48" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E48" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="F48">
         <v>4</v>
       </c>
       <c r="G48" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H48" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.15">
@@ -2634,22 +2653,22 @@
         <v>157</v>
       </c>
       <c r="C49" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D49" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="E49" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="F49">
         <v>4</v>
       </c>
       <c r="G49" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H49" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.15">
@@ -2672,10 +2691,10 @@
         <v>5</v>
       </c>
       <c r="G50" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H50" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.15">
@@ -2698,10 +2717,10 @@
         <v>6</v>
       </c>
       <c r="G51" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H51" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.15">
@@ -2724,10 +2743,10 @@
         <v>6</v>
       </c>
       <c r="G52" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H52" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.15">
@@ -2738,22 +2757,22 @@
         <v>156</v>
       </c>
       <c r="C53" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="D53" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="E53" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="F53">
         <v>5</v>
       </c>
       <c r="G53" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H53" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.15">
@@ -2776,10 +2795,10 @@
         <v>7</v>
       </c>
       <c r="G54" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H54" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.15">
@@ -2787,25 +2806,25 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C55" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="D55" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="E55" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="F55">
         <v>8</v>
       </c>
       <c r="G55" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H55" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.15">
@@ -2813,22 +2832,22 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C56" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="D56" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="E56" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="F56">
         <v>5</v>
       </c>
       <c r="G56" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.15">
@@ -2836,25 +2855,25 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C57" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D57" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="E57" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="F57">
         <v>3</v>
       </c>
       <c r="G57" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H57" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.15">
@@ -2862,25 +2881,25 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C58" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D58" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="E58" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="F58">
         <v>3</v>
       </c>
       <c r="G58" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H58" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.15">
@@ -2888,25 +2907,25 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C59" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="D59" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="E59" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="F59">
         <v>4</v>
       </c>
       <c r="G59" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H59" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.15">
@@ -2914,25 +2933,25 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C60" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="D60" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="E60" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="F60">
         <v>4</v>
       </c>
       <c r="G60" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H60" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.15">
@@ -2940,25 +2959,25 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C61" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="D61" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="E61" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="F61">
         <v>5</v>
       </c>
       <c r="G61" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H61" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.15">
@@ -2966,25 +2985,25 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C62" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D62" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E62" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="F62">
         <v>6</v>
       </c>
       <c r="G62" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H62" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.15">
@@ -2992,25 +3011,25 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
+        <v>194</v>
+      </c>
+      <c r="C63" t="s">
         <v>196</v>
       </c>
-      <c r="C63" t="s">
-        <v>198</v>
-      </c>
       <c r="D63" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E63" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F63">
         <v>6</v>
       </c>
       <c r="G63" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H63" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.15">
@@ -3018,25 +3037,25 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
+        <v>195</v>
+      </c>
+      <c r="C64" t="s">
         <v>197</v>
       </c>
-      <c r="C64" t="s">
-        <v>199</v>
-      </c>
       <c r="D64" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="E64" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F64">
         <v>7</v>
       </c>
       <c r="G64" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H64" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.15">
@@ -3044,25 +3063,25 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C65" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D65" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E65" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="F65">
         <v>6</v>
       </c>
       <c r="G65" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H65" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.15">
@@ -3070,25 +3089,25 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C66" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D66" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E66" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="F66">
         <v>6</v>
       </c>
       <c r="G66" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H66" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.15">
@@ -3096,25 +3115,25 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
+        <v>202</v>
+      </c>
+      <c r="C67" t="s">
         <v>204</v>
       </c>
-      <c r="C67" t="s">
-        <v>206</v>
-      </c>
       <c r="D67" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="E67" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F67">
         <v>6</v>
       </c>
       <c r="G67" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H67" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.15">
@@ -3122,25 +3141,25 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
+        <v>203</v>
+      </c>
+      <c r="C68" t="s">
         <v>205</v>
       </c>
-      <c r="C68" t="s">
-        <v>207</v>
-      </c>
       <c r="D68" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="E68" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F68">
         <v>6</v>
       </c>
       <c r="G68" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H68" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -3152,7 +3171,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -3381,10 +3400,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>57</v>
+        <v>286</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>58</v>
+        <v>287</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>59</v>
@@ -3537,7 +3556,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -3560,7 +3579,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -3583,7 +3602,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="4">
         <v>18</v>
       </c>
@@ -3609,7 +3628,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -3632,7 +3651,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="4">
         <v>20</v>
       </c>
@@ -3655,7 +3674,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -3678,7 +3697,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="4">
         <v>22</v>
       </c>
@@ -3701,7 +3720,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -3727,7 +3746,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="4">
         <v>24</v>
       </c>
@@ -3750,7 +3769,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -3773,7 +3792,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="5">
         <v>26</v>
       </c>
@@ -3796,7 +3815,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A28">
         <v>27</v>
       </c>
@@ -3818,11 +3837,8 @@
       <c r="H28" t="s">
         <v>155</v>
       </c>
-      <c r="I28" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.15">
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3845,7 +3861,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A30">
         <v>29</v>
       </c>
@@ -3868,7 +3884,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A31">
         <v>30</v>
       </c>
@@ -3891,7 +3907,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A32">
         <v>31</v>
       </c>
@@ -3914,7 +3930,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A33">
         <v>32</v>
       </c>
@@ -3937,7 +3953,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A34">
         <v>33</v>
       </c>
@@ -3957,7 +3973,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A35">
         <v>34</v>
       </c>
@@ -3980,7 +3996,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A36">
         <v>35</v>
       </c>
@@ -4000,7 +4016,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A37">
         <v>36</v>
       </c>
@@ -4020,7 +4036,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A38">
         <v>37</v>
       </c>
@@ -4040,7 +4056,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A39">
         <v>38</v>
       </c>
@@ -4057,10 +4073,10 @@
         <v>192</v>
       </c>
       <c r="F39" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.15">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A40">
         <v>39</v>
       </c>
@@ -4077,10 +4093,10 @@
         <v>191</v>
       </c>
       <c r="F40" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.15">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A41">
         <v>40</v>
       </c>
@@ -4097,177 +4113,171 @@
         <v>152</v>
       </c>
       <c r="F41" t="s">
-        <v>195</v>
-      </c>
-      <c r="I41" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.15">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" t="s">
+        <v>194</v>
+      </c>
+      <c r="C42" t="s">
+        <v>195</v>
+      </c>
+      <c r="D42" t="s">
         <v>196</v>
       </c>
-      <c r="C42" t="s">
+      <c r="E42" t="s">
         <v>197</v>
       </c>
-      <c r="D42" t="s">
+      <c r="F42" t="s">
         <v>198</v>
       </c>
-      <c r="E42" t="s">
+      <c r="H42" t="s">
         <v>199</v>
       </c>
-      <c r="F42" t="s">
-        <v>200</v>
-      </c>
-      <c r="H42" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.15">
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" t="s">
+        <v>195</v>
+      </c>
+      <c r="C43" t="s">
+        <v>194</v>
+      </c>
+      <c r="D43" t="s">
         <v>197</v>
       </c>
-      <c r="C43" t="s">
+      <c r="E43" t="s">
         <v>196</v>
       </c>
-      <c r="D43" t="s">
-        <v>199</v>
-      </c>
-      <c r="E43" t="s">
-        <v>198</v>
-      </c>
       <c r="F43" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H43" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.15">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" t="s">
+        <v>202</v>
+      </c>
+      <c r="C44" t="s">
+        <v>203</v>
+      </c>
+      <c r="D44" t="s">
         <v>204</v>
       </c>
-      <c r="C44" t="s">
+      <c r="E44" t="s">
         <v>205</v>
       </c>
-      <c r="D44" t="s">
+      <c r="F44" t="s">
+        <v>285</v>
+      </c>
+      <c r="H44" t="s">
         <v>206</v>
       </c>
-      <c r="E44" t="s">
-        <v>207</v>
-      </c>
-      <c r="F44" t="s">
-        <v>208</v>
-      </c>
-      <c r="H44" t="s">
-        <v>209</v>
-      </c>
-      <c r="I44" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.15">
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" t="s">
+        <v>207</v>
+      </c>
+      <c r="C45" t="s">
+        <v>208</v>
+      </c>
+      <c r="D45" t="s">
+        <v>209</v>
+      </c>
+      <c r="E45" t="s">
         <v>210</v>
       </c>
-      <c r="C45" t="s">
+      <c r="F45" t="s">
         <v>211</v>
       </c>
-      <c r="D45" t="s">
+      <c r="H45" t="s">
         <v>212</v>
       </c>
-      <c r="E45" t="s">
-        <v>213</v>
-      </c>
-      <c r="F45" t="s">
-        <v>214</v>
-      </c>
-      <c r="H45" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.15">
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C46" t="s">
+        <v>207</v>
+      </c>
+      <c r="D46" t="s">
         <v>210</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
+        <v>209</v>
+      </c>
+      <c r="F46" t="s">
         <v>213</v>
       </c>
-      <c r="E46" t="s">
+      <c r="H46" t="s">
         <v>212</v>
       </c>
-      <c r="F46" t="s">
-        <v>216</v>
-      </c>
-      <c r="H46" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.15">
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" t="s">
+        <v>214</v>
+      </c>
+      <c r="C47" t="s">
+        <v>215</v>
+      </c>
+      <c r="D47" t="s">
+        <v>216</v>
+      </c>
+      <c r="E47" t="s">
         <v>217</v>
       </c>
-      <c r="C47" t="s">
+      <c r="F47" t="s">
         <v>218</v>
       </c>
-      <c r="D47" t="s">
+      <c r="H47" t="s">
         <v>219</v>
       </c>
-      <c r="E47" t="s">
-        <v>220</v>
-      </c>
-      <c r="F47" t="s">
-        <v>221</v>
-      </c>
-      <c r="H47" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.15">
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C48" t="s">
+        <v>214</v>
+      </c>
+      <c r="D48" t="s">
         <v>217</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
+        <v>216</v>
+      </c>
+      <c r="F48" t="s">
         <v>220</v>
       </c>
-      <c r="E48" t="s">
+      <c r="G48" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="H48" t="s">
         <v>219</v>
-      </c>
-      <c r="F48" t="s">
-        <v>223</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="H48" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.15">
@@ -4275,19 +4285,19 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
+        <v>203</v>
+      </c>
+      <c r="C49" t="s">
+        <v>202</v>
+      </c>
+      <c r="D49" t="s">
         <v>205</v>
       </c>
-      <c r="C49" t="s">
+      <c r="E49" t="s">
         <v>204</v>
       </c>
-      <c r="D49" t="s">
-        <v>207</v>
-      </c>
-      <c r="E49" t="s">
-        <v>206</v>
-      </c>
       <c r="F49" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.15">
@@ -4295,19 +4305,19 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
+        <v>214</v>
+      </c>
+      <c r="C50" t="s">
+        <v>215</v>
+      </c>
+      <c r="D50" t="s">
+        <v>216</v>
+      </c>
+      <c r="E50" t="s">
         <v>217</v>
       </c>
-      <c r="C50" t="s">
-        <v>218</v>
-      </c>
-      <c r="D50" t="s">
-        <v>219</v>
-      </c>
-      <c r="E50" t="s">
-        <v>220</v>
-      </c>
       <c r="F50" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.15">
@@ -4315,19 +4325,19 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C51" t="s">
+        <v>214</v>
+      </c>
+      <c r="D51" t="s">
         <v>217</v>
       </c>
-      <c r="D51" t="s">
-        <v>220</v>
-      </c>
       <c r="E51" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="F51" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.15">
@@ -4335,19 +4345,19 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C52" t="s">
+        <v>214</v>
+      </c>
+      <c r="D52" t="s">
         <v>217</v>
       </c>
-      <c r="D52" t="s">
-        <v>220</v>
-      </c>
       <c r="E52" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="F52" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.15">
@@ -4355,19 +4365,19 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
+        <v>214</v>
+      </c>
+      <c r="C53" t="s">
+        <v>215</v>
+      </c>
+      <c r="D53" t="s">
+        <v>216</v>
+      </c>
+      <c r="E53" t="s">
         <v>217</v>
       </c>
-      <c r="C53" t="s">
-        <v>218</v>
-      </c>
-      <c r="D53" t="s">
-        <v>219</v>
-      </c>
-      <c r="E53" t="s">
-        <v>220</v>
-      </c>
       <c r="F53" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.15">
@@ -4387,10 +4397,70 @@
         <v>42</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="H54" s="4" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>203</v>
+      </c>
+      <c r="C55" t="s">
+        <v>202</v>
+      </c>
+      <c r="D55" t="s">
+        <v>205</v>
+      </c>
+      <c r="E55" t="s">
+        <v>204</v>
+      </c>
+      <c r="F55" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>100</v>
+      </c>
+      <c r="C56" t="s">
+        <v>99</v>
+      </c>
+      <c r="D56" t="s">
+        <v>102</v>
+      </c>
+      <c r="E56" t="s">
+        <v>101</v>
+      </c>
+      <c r="F56" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>